<commit_message>
Tag "Intent Token" COLLISION; refresh williams-intent-token to -02
Three unrelated drafts define an artifact named exactly "Intent Token":
williams-intent-token, haberkamp-ipp and chen-oauth-agent-intent-token.
Tagged on all three rows and recorded under COLLISION in CLAUDE.md, with
a note to search titles and summaries for a new draft's headline artifact
name, not just its acronym.

williams-intent-token: comment updated from -01 to -02 (5 Sep 2026); notes
the -01 additions (FIT, Authorization Fluidity, FCTG), that -02 is
editorial, and that the draft asserts a patent priority date (formal IPR
disclosure not verified).

Completed with the help of Claude
</commit_message>
<xml_diff>
--- a/delegated_authorization_research.xlsx
+++ b/delegated_authorization_research.xlsx
@@ -3585,7 +3585,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, 22 Jun 2026; author: Jeffrey Williams (Independent). Overlaps conceptually with draft-kroehl-agentic-trust-aae and draft-nelson-agent-delegation-receipts; worth tracking as a lighter-weight alternative to both.</t>
+          <t>Revision -02, 5 Sep 2026 (was -01, 22 Jun 2026; -00, 19 Mar 2026); author: Jeffrey Williams (Independent). **Updated 28 Oct 2026.** -01 added substantial machinery — Fractal Intent Token (FIT) binding for multi-scale agent systems, "Authorization Fluidity" for context-sensitive mode switching, and a Fractal Crypto-Temporal Graph (FCTG) as the normative audit-trail structure — so the row's original "lighter-weight alternative" framing (written at -01's filing) no longer fits well. -02 is editorial: it corrects the stated patent priority date, adds a fourth claimed instance of independent convergence (Broadcom's AgentMinder), and revises its account of AI-assisted development in Section 12. **Caveat: the draft text asserts a patent priority date**; whether a formal IPR disclosure is filed on Datatracker was not verified (the IPR search page sits behind a Cloudflare challenge). Overlaps conceptually with draft-kroehl-agentic-trust-aae and draft-nelson-agent-delegation-receipts. **COLLISION — "Intent Token" (tagged 28 Oct 2026):** three unrelated designs use this exact name — `williams-intent-token` (a human-declared authorization envelope bound to one action before it executes), `haberkamp-ipp` (a token that travels with every action through an agent chain carrying the verified original intent), and `chen-oauth-agent-intent-token` (an OAuth credential carrying the user's high-level intent so its translation into grants can be checked). Always name the full slug.</t>
         </is>
       </c>
     </row>
@@ -4515,7 +4515,7 @@
       </c>
       <c r="F118" s="5" t="inlineStr">
         <is>
-          <t>Revision -01, Jul 2026. Addresses the 'intent drift' threat class from draft-jiang-intent-security (corpus) with a concrete token artifact; complements the EMILIA Protocol receipts (authorization at the action level) with an intent record at the delegation chain level. The traveling Intent Token model is distinct from both SOOS Mandate JWTs (Sato, governance substrate) and McGuinness Actor Profiles (delegation chain encoding in existing OAuth tokens).</t>
+          <t>Revision -01, Jul 2026. Addresses the 'intent drift' threat class from draft-jiang-intent-security (corpus) with a concrete token artifact; complements the EMILIA Protocol receipts (authorization at the action level) with an intent record at the delegation chain level. The traveling Intent Token model is distinct from both SOOS Mandate JWTs (Sato, governance substrate) and McGuinness Actor Profiles (delegation chain encoding in existing OAuth tokens). **COLLISION — "Intent Token" (tagged 28 Oct 2026):** three unrelated designs use this exact name — `williams-intent-token` (a human-declared authorization envelope bound to one action before it executes), `haberkamp-ipp` (a token that travels with every action through an agent chain carrying the verified original intent), and `chen-oauth-agent-intent-token` (an OAuth credential carrying the user's high-level intent so its translation into grants can be checked). Always name the full slug.</t>
         </is>
       </c>
     </row>
@@ -15765,7 +15765,7 @@
       </c>
       <c r="F493" s="5" t="inlineStr">
         <is>
-          <t>Revision -00, 19 Oct 2026. **Added 28 Oct 2026 sweep.** China Mobile + Huawei. Introduced at the OAuth interim and followed up on the list (6-message thread). An Intent Token carrying the user's high-level intent so its translation into low-level grants can be checked. Same authors as the tracked `chen-oauth-agent-authz-use-cases`, whose "authorization context gap" this is meant to close.</t>
+          <t>Revision -00, 19 Oct 2026. **Added 28 Oct 2026 sweep.** China Mobile + Huawei. Introduced at the OAuth interim and followed up on the list (6-message thread). An Intent Token carrying the user's high-level intent so its translation into low-level grants can be checked. Same authors as the tracked `chen-oauth-agent-authz-use-cases`, whose "authorization context gap" this is meant to close. **COLLISION — "Intent Token" (tagged 28 Oct 2026):** three unrelated designs use this exact name — `williams-intent-token` (a human-declared authorization envelope bound to one action before it executes), `haberkamp-ipp` (a token that travels with every action through an agent chain carrying the verified original intent), and `chen-oauth-agent-intent-token` (an OAuth credential carrying the user's high-level intent so its translation into grants can be checked). Always name the full slug.</t>
         </is>
       </c>
     </row>

</xml_diff>